<commit_message>
Updated ITA_grids_kan model - 2025-12-12 14:13
</commit_message>
<xml_diff>
--- a/VerveStacks_ITA_grids_kan/ReportDefs_vervestacks.xlsx
+++ b/VerveStacks_ITA_grids_kan/ReportDefs_vervestacks.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Veda\Veda\Veda_models\vervestacks_models\VerveStacks_ITA_grids_kan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{26011915-674D-4311-B339-39DBD30E70E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{74C05D52-FE9C-4F03-A982-2ED8C40F4A0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4978,7 +4978,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DF3C4D3E-0D7C-4362-9273-0F727F1A0EF1}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54BB984A-03BD-4CE6-B952-13AD4D97D7A6}">
   <dimension ref="B9:H337"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>
@@ -35098,7 +35098,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1A5314C3-5775-423A-A881-11043BBE7EA3}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73D790EB-4D74-44B0-9F24-9555924805B5}">
   <dimension ref="B9:L337"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <sheetData>

</xml_diff>